<commit_message>
figured out list-ception issue
Fixed the headache from yesterday when I was trying to use nested pandas dataframes that was causing memory allocation issues.

Pivoted to using lists with my version of c++ structs, so I rewrote a ton of code to switch to the new data structure

Note to self, still a lot of logic issues but at least the data structure part seems to be working as intended
</commit_message>
<xml_diff>
--- a/VPD PO download generator/VPD PO Download Spreadsheet V0.1.xlsx
+++ b/VPD PO download generator/VPD PO Download Spreadsheet V0.1.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jwa25\source\repos\VPD PO download generator\VPD PO download generator\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C99DA321-4198-43EE-BEBE-E07807382B58}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5BC1522F-3E4A-4485-BA21-F159EB7D1E76}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{E1429B42-6D56-496D-8C3D-7089E84A1C10}"/>
+    <workbookView xWindow="-3195" yWindow="2760" windowWidth="21585" windowHeight="12765" xr2:uid="{E1429B42-6D56-496D-8C3D-7089E84A1C10}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="32" uniqueCount="25">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="32" uniqueCount="26">
   <si>
     <t>Type</t>
   </si>
@@ -101,6 +101,9 @@
   </si>
   <si>
     <t>Black/Black</t>
+  </si>
+  <si>
+    <t>R-SO-5106483-1-2</t>
   </si>
 </sst>
 </file>
@@ -492,6 +495,7 @@
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="20.5703125" customWidth="1"/>
+    <col min="2" max="2" width="20.42578125" customWidth="1"/>
     <col min="3" max="3" width="13.85546875" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="12.85546875" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="8.5703125" customWidth="1"/>
@@ -554,7 +558,7 @@
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>14</v>
+        <v>25</v>
       </c>
       <c r="B3" t="s">
         <v>9</v>

</xml_diff>

<commit_message>
stuff is functioning :')
Working on tying code together. Code so far seems to be working properly.

 So far:
  -Breaks out orders into necessary components (haven't done transom stuff yet)
  -Adds it into lists
  -Combines the first unit into the BOTH list. Need to make this work for all units in single list, not just the first one
</commit_message>
<xml_diff>
--- a/VPD PO download generator/VPD PO Download Spreadsheet V0.1.xlsx
+++ b/VPD PO download generator/VPD PO Download Spreadsheet V0.1.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jwa25\source\repos\VPD PO download generator\VPD PO download generator\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5BC1522F-3E4A-4485-BA21-F159EB7D1E76}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{22ACB638-831E-40B7-91A4-4CAFBD89C91C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-3195" yWindow="2760" windowWidth="21585" windowHeight="12765" xr2:uid="{E1429B42-6D56-496D-8C3D-7089E84A1C10}"/>
+    <workbookView xWindow="-16275" yWindow="4635" windowWidth="14040" windowHeight="9375" xr2:uid="{E1429B42-6D56-496D-8C3D-7089E84A1C10}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="32" uniqueCount="26">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="37" uniqueCount="27">
   <si>
     <t>Type</t>
   </si>
@@ -104,6 +104,9 @@
   </si>
   <si>
     <t>R-SO-5106483-1-2</t>
+  </si>
+  <si>
+    <t>R-SO-5106483-1-3</t>
   </si>
 </sst>
 </file>
@@ -491,7 +494,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3E0080E7-F391-47B1-85B3-22F42F81BBBC}">
-  <dimension ref="A1:H3"/>
+  <dimension ref="A1:H4"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="20.5703125" customWidth="1"/>
@@ -579,6 +582,32 @@
         <v>46091</v>
       </c>
       <c r="H3" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>26</v>
+      </c>
+      <c r="B4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C4">
+        <v>71.5</v>
+      </c>
+      <c r="D4">
+        <v>95.5</v>
+      </c>
+      <c r="E4" t="s">
+        <v>21</v>
+      </c>
+      <c r="F4" t="s">
+        <v>15</v>
+      </c>
+      <c r="G4" s="4">
+        <v>46091</v>
+      </c>
+      <c r="H4" t="s">
         <v>16</v>
       </c>
     </row>

</xml_diff>

<commit_message>
my mind is FRIED
🤯
</commit_message>
<xml_diff>
--- a/VPD PO download generator/VPD PO Download Spreadsheet V0.1.xlsx
+++ b/VPD PO download generator/VPD PO Download Spreadsheet V0.1.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jwa25\source\repos\VPD PO download generator\VPD PO download generator\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C1BFD1A9-D6E7-4873-B140-1A2C18555C39}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{910116DF-DD79-4D18-8522-40D29A76DFEB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="14303" yWindow="2595" windowWidth="21795" windowHeight="12975" xr2:uid="{E1429B42-6D56-496D-8C3D-7089E84A1C10}"/>
   </bookViews>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="57" uniqueCount="31">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="97" uniqueCount="39">
   <si>
     <t>Type</t>
   </si>
@@ -119,6 +119,30 @@
   </si>
   <si>
     <t>R-SO-5088990-1-7</t>
+  </si>
+  <si>
+    <t>R-SO-5088990-1-11</t>
+  </si>
+  <si>
+    <t>R-SO-5088990-1-12</t>
+  </si>
+  <si>
+    <t>R-SO-5088990-1-13</t>
+  </si>
+  <si>
+    <t>R-SO-5088990-1-14</t>
+  </si>
+  <si>
+    <t>R-SO-5088990-1-15</t>
+  </si>
+  <si>
+    <t>R-SO-5088990-1-16</t>
+  </si>
+  <si>
+    <t>R-SO-5088990-1-17</t>
+  </si>
+  <si>
+    <t>R-SO-5088990-1-18</t>
   </si>
 </sst>
 </file>
@@ -512,7 +536,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3E0080E7-F391-47B1-85B3-22F42F81BBBC}">
-  <dimension ref="A1:H8"/>
+  <dimension ref="A1:H16"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="20.5703125" customWidth="1"/>
@@ -730,6 +754,214 @@
         <v>46007</v>
       </c>
       <c r="H8" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>31</v>
+      </c>
+      <c r="B9" t="s">
+        <v>9</v>
+      </c>
+      <c r="C9">
+        <v>71.5</v>
+      </c>
+      <c r="D9">
+        <v>79.5</v>
+      </c>
+      <c r="E9" t="s">
+        <v>17</v>
+      </c>
+      <c r="F9" t="s">
+        <v>14</v>
+      </c>
+      <c r="G9" s="4">
+        <v>46007</v>
+      </c>
+      <c r="H9" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="10" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>32</v>
+      </c>
+      <c r="B10" t="s">
+        <v>9</v>
+      </c>
+      <c r="C10">
+        <v>71.5</v>
+      </c>
+      <c r="D10">
+        <v>79.5</v>
+      </c>
+      <c r="E10" t="s">
+        <v>17</v>
+      </c>
+      <c r="F10" t="s">
+        <v>14</v>
+      </c>
+      <c r="G10" s="4">
+        <v>46007</v>
+      </c>
+      <c r="H10" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="11" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>33</v>
+      </c>
+      <c r="B11" t="s">
+        <v>9</v>
+      </c>
+      <c r="C11">
+        <v>71.5</v>
+      </c>
+      <c r="D11">
+        <v>79.5</v>
+      </c>
+      <c r="E11" t="s">
+        <v>17</v>
+      </c>
+      <c r="F11" t="s">
+        <v>14</v>
+      </c>
+      <c r="G11" s="4">
+        <v>46007</v>
+      </c>
+      <c r="H11" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="12" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>34</v>
+      </c>
+      <c r="B12" t="s">
+        <v>9</v>
+      </c>
+      <c r="C12">
+        <v>71.5</v>
+      </c>
+      <c r="D12">
+        <v>79.5</v>
+      </c>
+      <c r="E12" t="s">
+        <v>17</v>
+      </c>
+      <c r="F12" t="s">
+        <v>14</v>
+      </c>
+      <c r="G12" s="4">
+        <v>46007</v>
+      </c>
+      <c r="H12" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="13" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>35</v>
+      </c>
+      <c r="B13" t="s">
+        <v>9</v>
+      </c>
+      <c r="C13">
+        <v>71.5</v>
+      </c>
+      <c r="D13">
+        <v>79.5</v>
+      </c>
+      <c r="E13" t="s">
+        <v>17</v>
+      </c>
+      <c r="F13" t="s">
+        <v>14</v>
+      </c>
+      <c r="G13" s="4">
+        <v>46007</v>
+      </c>
+      <c r="H13" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="14" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
+        <v>36</v>
+      </c>
+      <c r="B14" t="s">
+        <v>9</v>
+      </c>
+      <c r="C14">
+        <v>59.5</v>
+      </c>
+      <c r="D14">
+        <v>79.5</v>
+      </c>
+      <c r="E14" t="s">
+        <v>17</v>
+      </c>
+      <c r="F14" t="s">
+        <v>14</v>
+      </c>
+      <c r="G14" s="4">
+        <v>46007</v>
+      </c>
+      <c r="H14" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="15" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
+        <v>37</v>
+      </c>
+      <c r="B15" t="s">
+        <v>9</v>
+      </c>
+      <c r="C15">
+        <v>59.5</v>
+      </c>
+      <c r="D15">
+        <v>79.5</v>
+      </c>
+      <c r="E15" t="s">
+        <v>17</v>
+      </c>
+      <c r="F15" t="s">
+        <v>14</v>
+      </c>
+      <c r="G15" s="4">
+        <v>46007</v>
+      </c>
+      <c r="H15" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="16" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
+        <v>38</v>
+      </c>
+      <c r="B16" t="s">
+        <v>9</v>
+      </c>
+      <c r="C16">
+        <v>59.5</v>
+      </c>
+      <c r="D16">
+        <v>79.5</v>
+      </c>
+      <c r="E16" t="s">
+        <v>17</v>
+      </c>
+      <c r="F16" t="s">
+        <v>14</v>
+      </c>
+      <c r="G16" s="4">
+        <v>46008</v>
+      </c>
+      <c r="H16" t="s">
         <v>15</v>
       </c>
     </row>

</xml_diff>